<commit_message>
fix: corrige formulas e valores de alocacao e salario na planilha
</commit_message>
<xml_diff>
--- a/investment_simulator.xlsx
+++ b/investment_simulator.xlsx
@@ -43,12 +43,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
@@ -89,18 +89,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,32 +498,32 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="3" t="n">
         <v>2000</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Rendimento Carteira</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="4" t="n">
         <v>0.006</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Sugestão de Investimento (30%)</t>
         </is>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <f>D10*0.3</f>
         <v/>
       </c>
@@ -536,54 +537,54 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Quanto investir por mês ?</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="3" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Por Quantos Anos ?</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Taxa de Rendimento mensal ?</t>
         </is>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="5">
         <f>D11</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Patrimônio acumulado ?</t>
         </is>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <f>VF(D17; D16*12; -D15)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Retorno Mensal Estimado ?</t>
         </is>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <f>D18*D11</f>
         <v/>
       </c>
@@ -597,83 +598,83 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Anos</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Patrimônio Acumulado</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Retorno Mensal Estimado</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <f>VF($D$17; B23*12; -$D$15)</f>
         <v/>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <f>C23*$D$17</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <f>VF($D$17; B24*12; -$D$15)</f>
         <v/>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <f>C24*$D$17</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <f>VF($D$17; B25*12; -$D$15)</f>
         <v/>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <f>C25*$D$17</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <f>VF($D$17; B26*12; -$D$15)</f>
         <v/>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="3">
         <f>C26*$D$17</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="3">
         <f>VF($D$17; B27*12; -$D$15)</f>
         <v/>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="3">
         <f>C27*$D$17</f>
         <v/>
       </c>
@@ -711,108 +712,108 @@
     </row>
     <row r="32"/>
     <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>TIPO DE INVESTIMENTO</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Percentual Sugerido</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Valores (R$)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
       </c>
-      <c r="C34" s="5">
+      <c r="C34" s="4">
         <f>PROCX($C$30 &amp; "-" &amp; B34; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
         <v/>
       </c>
-      <c r="D34" s="4">
+      <c r="D34" s="3">
         <f>C34*$C$31</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="C35" s="5">
+      <c r="C35" s="4">
         <f>PROCX($C$30 &amp; "-" &amp; B35; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
         <v/>
       </c>
-      <c r="D35" s="4">
+      <c r="D35" s="3">
         <f>C35*$C$31</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
       </c>
-      <c r="C36" s="5">
+      <c r="C36" s="4">
         <f>PROCX($C$30 &amp; "-" &amp; B36; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
         <v/>
       </c>
-      <c r="D36" s="4">
+      <c r="D36" s="3">
         <f>C36*$C$31</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="4">
         <f>PROCX($C$30 &amp; "-" &amp; B37; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
         <v/>
       </c>
-      <c r="D37" s="4">
+      <c r="D37" s="3">
         <f>C37*$C$31</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
       </c>
-      <c r="C38" s="5">
+      <c r="C38" s="4">
         <f>PROCX($C$30 &amp; "-" &amp; B38; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
         <v/>
       </c>
-      <c r="D38" s="4">
+      <c r="D38" s="3">
         <f>C38*$C$31</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="C39" s="5">
+      <c r="C39" s="4">
         <f>PROCX($C$30 &amp; "-" &amp; B39; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
         <v/>
       </c>
-      <c r="D39" s="4">
+      <c r="D39" s="3">
         <f>C39*$C$31</f>
         <v/>
       </c>
@@ -847,7 +848,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -875,362 +876,362 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Conservador-RENDA FIXA</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="11" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Conservador-IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="11" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Conservador-MULTIMERCADO</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="11" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Conservador-AÇÕES BR</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="11" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Conservador-INTERNACIONAL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Conservador-CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Moderado-RENDA FIXA</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="11" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Moderado-IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="11" t="n">
         <v>0.32</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Moderado-MULTIMERCADO</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="11" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Moderado-AÇÕES BR</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="11" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Moderado-INTERNACIONAL</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="11" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Moderado-CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="11" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Agressivo-RENDA FIXA</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="11" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Agressivo-IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="11" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Agressivo-MULTIMERCADO</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="11" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Agressivo-AÇÕES BR</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="11" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Agressivo-INTERNACIONAL</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="11" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Agressivo-CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Agressivo</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>CRIPTOMOEDAS</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="n">
         <v>0.1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: atualiza script com logica 100% dinamica via PROCX
</commit_message>
<xml_diff>
--- a/investment_simulator.xlsx
+++ b/investment_simulator.xlsx
@@ -49,11 +49,11 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -98,10 +98,10 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,7 +615,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="7" t="n">
+      <c r="B23" t="n">
         <v>2</v>
       </c>
       <c r="C23" s="3">
@@ -628,7 +628,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="7" t="n">
+      <c r="B24" t="n">
         <v>5</v>
       </c>
       <c r="C24" s="3">
@@ -641,7 +641,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="7" t="n">
+      <c r="B25" t="n">
         <v>10</v>
       </c>
       <c r="C25" s="3">
@@ -654,7 +654,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="7" t="n">
+      <c r="B26" t="n">
         <v>20</v>
       </c>
       <c r="C26" s="3">
@@ -667,7 +667,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="7" t="n">
+      <c r="B27" t="n">
         <v>30</v>
       </c>
       <c r="C27" s="3">
@@ -693,7 +693,7 @@
           <t>PERFIL SELECIONADO</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
@@ -705,7 +705,7 @@
           <t>VALOR A SER INVESTIDO POR MÊS</t>
         </is>
       </c>
-      <c r="C31" s="9">
+      <c r="C31" s="8">
         <f>D15</f>
         <v/>
       </c>
@@ -729,7 +729,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
@@ -744,7 +744,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
@@ -759,7 +759,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
@@ -774,7 +774,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
@@ -789,7 +789,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
@@ -804,7 +804,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
@@ -819,7 +819,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -828,7 +828,7 @@
         <f>SOMA(C34:C39)</f>
         <v/>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="8">
         <f>SOMA(D34:D39)</f>
         <v/>
       </c>
@@ -848,7 +848,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -876,17 +876,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Conservador-RENDA FIXA</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
@@ -896,17 +896,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Conservador-IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
@@ -916,17 +916,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Conservador-MULTIMERCADO</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
@@ -936,17 +936,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Conservador-AÇÕES BR</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
@@ -956,17 +956,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Conservador-INTERNACIONAL</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
@@ -976,17 +976,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Conservador-CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Conservador</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
@@ -996,17 +996,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Moderado-RENDA FIXA</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
@@ -1016,17 +1016,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Moderado-IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
@@ -1036,17 +1036,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Moderado-MULTIMERCADO</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
@@ -1056,17 +1056,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Moderado-AÇÕES BR</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
@@ -1076,17 +1076,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Moderado-INTERNACIONAL</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
@@ -1096,17 +1096,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Moderado-CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>
@@ -1116,17 +1116,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Agressivo-RENDA FIXA</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>RENDA FIXA</t>
         </is>
@@ -1136,17 +1136,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Agressivo-IMOBILIÁRIO</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>IMOBILIÁRIO</t>
         </is>
@@ -1156,17 +1156,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Agressivo-MULTIMERCADO</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>MULTIMERCADO</t>
         </is>
@@ -1176,17 +1176,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Agressivo-AÇÕES BR</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>AÇÕES BR</t>
         </is>
@@ -1196,17 +1196,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Agressivo-INTERNACIONAL</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Agressivo</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>INTERNACIONAL</t>
         </is>
@@ -1216,17 +1216,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Agressivo-CRIPTOMOEDAS</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>CRIPTOMOEDAS</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Agressivo</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>CRIPTOMOEDAS</t>
         </is>

</xml_diff>

<commit_message>
docs: adiciona README.md documentando a arquitetura modular com Gemini, spec.md e ajustes finais do simulador
</commit_message>
<xml_diff>
--- a/investment_simulator.xlsx
+++ b/investment_simulator.xlsx
@@ -48,12 +48,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -95,12 +95,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -467,20 +467,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="92" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="94" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="94" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>SIMULADOR DE INVESTIMENTOS</t>
+          <t>SIMULADOR DE INVESTIMENTOS MULTICLASSE</t>
         </is>
       </c>
     </row>
@@ -493,14 +494,14 @@
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>CONFIGURAÇÕES</t>
+          <t>1. CONFIGURAÇÕES GLOBAIS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>Salário</t>
+          <t>Salário Base</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -510,332 +511,346 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rendimento Carteira</t>
+          <t>Taxa Poupança Sugerida</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.006</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sugestão de Investimento (30%)</t>
+          <t>Sugestão de Aporte Mensal (30%)</t>
         </is>
       </c>
       <c r="D12" s="3">
-        <f>D10*0.3</f>
+        <f>D10*D11</f>
         <v/>
       </c>
     </row>
     <row r="13"/>
-    <row r="14">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>INVESTIMENTO MENSAL</t>
-        </is>
-      </c>
-    </row>
+    <row r="14"/>
     <row r="15">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Quanto investir por mês ?</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>200</v>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2. SELEÇÃO DE PERFIL E APORTE</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>Por Quantos Anos ?</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>5</v>
+          <t>Perfil de Investimento</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>Taxa de Rendimento mensal ?</t>
-        </is>
-      </c>
-      <c r="D17" s="5">
-        <f>D11</f>
+          <t>Valor Efetivo Aportado por Mês</t>
+        </is>
+      </c>
+      <c r="D17" s="6">
+        <f>D12</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>Patrimônio acumulado ?</t>
-        </is>
-      </c>
-      <c r="D18" s="3">
-        <f>VF(D17; D16*12; -D15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Retorno Mensal Estimado ?</t>
-        </is>
-      </c>
-      <c r="D19" s="3">
-        <f>D18*D11</f>
-        <v/>
-      </c>
-    </row>
+          <t>Taxa de Retorno Média da Carteira (a.m.)</t>
+        </is>
+      </c>
+      <c r="D18" s="7">
+        <f>SUMPRODUCT(C24:C29, E24:E29) / 12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20"/>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Cenários (Projeção de Longo Prazo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Anos</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Patrimônio Acumulado</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Retorno Mensal Estimado</t>
-        </is>
-      </c>
-    </row>
+          <t>3. DISTRIBUIÇÃO DA CARTEIRA POR ATIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
-      <c r="B23" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" s="3">
-        <f>VF($D$17; B23*12; -$D$15)</f>
-        <v/>
-      </c>
-      <c r="D23" s="3">
-        <f>C23*$D$17</f>
-        <v/>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>TIPO DE INVESTIMENTO</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Percentual na Carteira</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Aporte Alocado (R$)</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Retorno Esperado (a.a.)</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" t="n">
-        <v>5</v>
-      </c>
-      <c r="C24" s="3">
-        <f>VF($D$17; B24*12; -$D$15)</f>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>RENDA FIXA</t>
+        </is>
+      </c>
+      <c r="C24" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B24, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
         <v/>
       </c>
       <c r="D24" s="3">
         <f>C24*$D$17</f>
         <v/>
       </c>
+      <c r="E24" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B24, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
-      <c r="B25" t="n">
-        <v>10</v>
-      </c>
-      <c r="C25" s="3">
-        <f>VF($D$17; B25*12; -$D$15)</f>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>IMOBILIÁRIO</t>
+        </is>
+      </c>
+      <c r="C25" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B25, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
         <v/>
       </c>
       <c r="D25" s="3">
         <f>C25*$D$17</f>
         <v/>
       </c>
+      <c r="E25" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B25, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
-      <c r="B26" t="n">
-        <v>20</v>
-      </c>
-      <c r="C26" s="3">
-        <f>VF($D$17; B26*12; -$D$15)</f>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>MULTIMERCADO</t>
+        </is>
+      </c>
+      <c r="C26" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B26, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
         <v/>
       </c>
       <c r="D26" s="3">
         <f>C26*$D$17</f>
         <v/>
       </c>
+      <c r="E26" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B26, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
-      <c r="B27" t="n">
-        <v>30</v>
-      </c>
-      <c r="C27" s="3">
-        <f>VF($D$17; B27*12; -$D$15)</f>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>AÇÕES BR</t>
+        </is>
+      </c>
+      <c r="C27" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B27, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
         <v/>
       </c>
       <c r="D27" s="3">
         <f>C27*$D$17</f>
         <v/>
       </c>
-    </row>
-    <row r="28"/>
+      <c r="E27" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B27, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>INTERNACIONAL</t>
+        </is>
+      </c>
+      <c r="C28" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B28, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <v/>
+      </c>
+      <c r="D28" s="3">
+        <f>C28*$D$17</f>
+        <v/>
+      </c>
+      <c r="E28" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B28, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <v/>
+      </c>
+    </row>
     <row r="29">
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>DISTRIBUIÇÃO DE CARTEIRA POR PERFIL</t>
-        </is>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>CRIPTOMOEDAS</t>
+        </is>
+      </c>
+      <c r="C29" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B29, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <v/>
+      </c>
+      <c r="D29" s="3">
+        <f>C29*$D$17</f>
+        <v/>
+      </c>
+      <c r="E29" s="4">
+        <f>XLOOKUP($C$16 &amp; "-" &amp; B29, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>PERFIL SELECIONADO</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Moderado</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>VALOR A SER INVESTIDO POR MÊS</t>
-        </is>
-      </c>
-      <c r="C31" s="8">
-        <f>D15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C30" s="10">
+        <f>SUM(C24:C29)</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>SUM(D24:D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>4. PROJEÇÕES DE LONGO PRAZO (CENÁRIOS)</t>
+        </is>
+      </c>
+    </row>
     <row r="33">
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>TIPO DE INVESTIMENTO</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Percentual Sugerido</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Valores (R$)</t>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Anos</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Total Aportado (Capital)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Patrimônio Acumulado (com Juros)</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Rendimento Mensal Estimado</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>RENDA FIXA</t>
-        </is>
-      </c>
-      <c r="C34" s="4">
-        <f>PROCX($C$30 &amp; "-" &amp; B34; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="3">
+        <f>$D$17*2*12</f>
         <v/>
       </c>
       <c r="D34" s="3">
-        <f>C34*$C$31</f>
+        <f>FV($D$18, B34*12, -$D$17)</f>
+        <v/>
+      </c>
+      <c r="E34" s="3">
+        <f>D34*$D$18</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>IMOBILIÁRIO</t>
-        </is>
-      </c>
-      <c r="C35" s="4">
-        <f>PROCX($C$30 &amp; "-" &amp; B35; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
+      <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="3">
+        <f>$D$17*5*12</f>
         <v/>
       </c>
       <c r="D35" s="3">
-        <f>C35*$C$31</f>
+        <f>FV($D$18, B35*12, -$D$17)</f>
+        <v/>
+      </c>
+      <c r="E35" s="3">
+        <f>D35*$D$18</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>MULTIMERCADO</t>
-        </is>
-      </c>
-      <c r="C36" s="4">
-        <f>PROCX($C$30 &amp; "-" &amp; B36; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
+      <c r="B36" t="n">
+        <v>10</v>
+      </c>
+      <c r="C36" s="3">
+        <f>$D$17*10*12</f>
         <v/>
       </c>
       <c r="D36" s="3">
-        <f>C36*$C$31</f>
+        <f>FV($D$18, B36*12, -$D$17)</f>
+        <v/>
+      </c>
+      <c r="E36" s="3">
+        <f>D36*$D$18</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>AÇÕES BR</t>
-        </is>
-      </c>
-      <c r="C37" s="4">
-        <f>PROCX($C$30 &amp; "-" &amp; B37; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
+      <c r="B37" t="n">
+        <v>20</v>
+      </c>
+      <c r="C37" s="3">
+        <f>$D$17*20*12</f>
         <v/>
       </c>
       <c r="D37" s="3">
-        <f>C37*$C$31</f>
+        <f>FV($D$18, B37*12, -$D$17)</f>
+        <v/>
+      </c>
+      <c r="E37" s="3">
+        <f>D37*$D$18</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>INTERNACIONAL</t>
-        </is>
-      </c>
-      <c r="C38" s="4">
-        <f>PROCX($C$30 &amp; "-" &amp; B38; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
+      <c r="B38" t="n">
+        <v>30</v>
+      </c>
+      <c r="C38" s="3">
+        <f>$D$17*30*12</f>
         <v/>
       </c>
       <c r="D38" s="3">
-        <f>C38*$C$31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>CRIPTOMOEDAS</t>
-        </is>
-      </c>
-      <c r="C39" s="4">
-        <f>PROCX($C$30 &amp; "-" &amp; B39; Database_Profiles!$A$2:$A$19; Database_Profiles!$D$2:$D$19; 0)</f>
-        <v/>
-      </c>
-      <c r="D39" s="3">
-        <f>C39*$C$31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C40" s="10">
-        <f>SOMA(C34:C39)</f>
-        <v/>
-      </c>
-      <c r="D40" s="8">
-        <f>SOMA(D34:D39)</f>
+        <f>FV($D$18, B38*12, -$D$17)</f>
+        <v/>
+      </c>
+      <c r="E38" s="3">
+        <f>D38*$D$18</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Database_Profiles!$F$2:$F$4</formula1>
     </dataValidation>
   </dataValidations>
@@ -856,7 +871,7 @@
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -881,6 +896,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>RETORNO AA</t>
+        </is>
+      </c>
       <c r="F1" t="inlineStr">
         <is>
           <t>Perfis_Unicos</t>
@@ -906,6 +926,9 @@
       <c r="D2" s="11" t="n">
         <v>0.5</v>
       </c>
+      <c r="E2" s="11" t="n">
+        <v>0.1</v>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Conservador</t>
@@ -931,6 +954,9 @@
       <c r="D3" s="11" t="n">
         <v>0.3</v>
       </c>
+      <c r="E3" s="11" t="n">
+        <v>0.11</v>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Moderado</t>
@@ -956,6 +982,9 @@
       <c r="D4" s="11" t="n">
         <v>0.1</v>
       </c>
+      <c r="E4" s="11" t="n">
+        <v>0.105</v>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Agressivo</t>
@@ -981,6 +1010,9 @@
       <c r="D5" s="11" t="n">
         <v>0.1</v>
       </c>
+      <c r="E5" s="11" t="n">
+        <v>0.12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1001,6 +1033,9 @@
       <c r="D6" s="11" t="n">
         <v>0</v>
       </c>
+      <c r="E6" s="11" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1021,6 +1056,9 @@
       <c r="D7" s="11" t="n">
         <v>0</v>
       </c>
+      <c r="E7" s="11" t="n">
+        <v>0.18</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1041,6 +1079,9 @@
       <c r="D8" s="11" t="n">
         <v>0.35</v>
       </c>
+      <c r="E8" s="11" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1061,6 +1102,9 @@
       <c r="D9" s="11" t="n">
         <v>0.32</v>
       </c>
+      <c r="E9" s="11" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1081,6 +1125,9 @@
       <c r="D10" s="11" t="n">
         <v>0.08</v>
       </c>
+      <c r="E10" s="11" t="n">
+        <v>0.105</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -1101,6 +1148,9 @@
       <c r="D11" s="11" t="n">
         <v>0.1</v>
       </c>
+      <c r="E11" s="11" t="n">
+        <v>0.12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1121,6 +1171,9 @@
       <c r="D12" s="11" t="n">
         <v>0.1</v>
       </c>
+      <c r="E12" s="11" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1141,6 +1194,9 @@
       <c r="D13" s="11" t="n">
         <v>0.05</v>
       </c>
+      <c r="E13" s="11" t="n">
+        <v>0.18</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1161,6 +1217,9 @@
       <c r="D14" s="11" t="n">
         <v>0.1</v>
       </c>
+      <c r="E14" s="11" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1181,6 +1240,9 @@
       <c r="D15" s="11" t="n">
         <v>0.2</v>
       </c>
+      <c r="E15" s="11" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -1201,6 +1263,9 @@
       <c r="D16" s="11" t="n">
         <v>0.05</v>
       </c>
+      <c r="E16" s="11" t="n">
+        <v>0.105</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -1221,6 +1286,9 @@
       <c r="D17" s="11" t="n">
         <v>0.35</v>
       </c>
+      <c r="E17" s="11" t="n">
+        <v>0.12</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1241,6 +1309,9 @@
       <c r="D18" s="11" t="n">
         <v>0.2</v>
       </c>
+      <c r="E18" s="11" t="n">
+        <v>0.115</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1260,6 +1331,9 @@
       </c>
       <c r="D19" s="11" t="n">
         <v>0.1</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>0.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: atualiza fórmulas para PROCV e padrão brasileiro em português
</commit_message>
<xml_diff>
--- a/investment_simulator.xlsx
+++ b/investment_simulator.xlsx
@@ -472,9 +472,9 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="94" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="94" customWidth="1" min="5" max="5"/>
+    <col width="69" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="69" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="D18" s="7">
-        <f>SUMPRODUCT(C24:C29, E24:E29) / 12</f>
+        <f>SOMAPRODUTO(C24:C29; E24:E29) / 12</f>
         <v/>
       </c>
     </row>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C24" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B24, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B24; Database_Profiles!$A$2:$E$19; 4; FALSO)</f>
         <v/>
       </c>
       <c r="D24" s="3">
@@ -619,7 +619,7 @@
         <v/>
       </c>
       <c r="E24" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B24, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B24; Database_Profiles!$A$2:$E$19; 5; FALSO)</f>
         <v/>
       </c>
     </row>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="C25" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B25, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B25; Database_Profiles!$A$2:$E$19; 4; FALSO)</f>
         <v/>
       </c>
       <c r="D25" s="3">
@@ -638,7 +638,7 @@
         <v/>
       </c>
       <c r="E25" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B25, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B25; Database_Profiles!$A$2:$E$19; 5; FALSO)</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="C26" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B26, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B26; Database_Profiles!$A$2:$E$19; 4; FALSO)</f>
         <v/>
       </c>
       <c r="D26" s="3">
@@ -657,7 +657,7 @@
         <v/>
       </c>
       <c r="E26" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B26, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B26; Database_Profiles!$A$2:$E$19; 5; FALSO)</f>
         <v/>
       </c>
     </row>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="C27" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B27, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B27; Database_Profiles!$A$2:$E$19; 4; FALSO)</f>
         <v/>
       </c>
       <c r="D27" s="3">
@@ -676,7 +676,7 @@
         <v/>
       </c>
       <c r="E27" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B27, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B27; Database_Profiles!$A$2:$E$19; 5; FALSO)</f>
         <v/>
       </c>
     </row>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="C28" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B28, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B28; Database_Profiles!$A$2:$E$19; 4; FALSO)</f>
         <v/>
       </c>
       <c r="D28" s="3">
@@ -695,7 +695,7 @@
         <v/>
       </c>
       <c r="E28" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B28, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B28; Database_Profiles!$A$2:$E$19; 5; FALSO)</f>
         <v/>
       </c>
     </row>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="C29" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B29, Database_Profiles!$A$2:$A$19, Database_Profiles!$D$2:$D$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B29; Database_Profiles!$A$2:$E$19; 4; FALSO)</f>
         <v/>
       </c>
       <c r="D29" s="3">
@@ -714,7 +714,7 @@
         <v/>
       </c>
       <c r="E29" s="4">
-        <f>XLOOKUP($C$16 &amp; "-" &amp; B29, Database_Profiles!$A$2:$A$19, Database_Profiles!$E$2:$E$19, 0)</f>
+        <f>PROCV($C$16 &amp; "-" &amp; B29; Database_Profiles!$A$2:$E$19; 5; FALSO)</f>
         <v/>
       </c>
     </row>
@@ -725,11 +725,11 @@
         </is>
       </c>
       <c r="C30" s="10">
-        <f>SUM(C24:C29)</f>
+        <f>SOMA(C24:C29)</f>
         <v/>
       </c>
       <c r="D30" s="6">
-        <f>SUM(D24:D29)</f>
+        <f>SOMA(D24:D29)</f>
         <v/>
       </c>
     </row>
@@ -772,7 +772,7 @@
         <v/>
       </c>
       <c r="D34" s="3">
-        <f>FV($D$18, B34*12, -$D$17)</f>
+        <f>VF($D$18; B34*12; -$D$17)</f>
         <v/>
       </c>
       <c r="E34" s="3">
@@ -789,7 +789,7 @@
         <v/>
       </c>
       <c r="D35" s="3">
-        <f>FV($D$18, B35*12, -$D$17)</f>
+        <f>VF($D$18; B35*12; -$D$17)</f>
         <v/>
       </c>
       <c r="E35" s="3">
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="D36" s="3">
-        <f>FV($D$18, B36*12, -$D$17)</f>
+        <f>VF($D$18; B36*12; -$D$17)</f>
         <v/>
       </c>
       <c r="E36" s="3">
@@ -823,7 +823,7 @@
         <v/>
       </c>
       <c r="D37" s="3">
-        <f>FV($D$18, B37*12, -$D$17)</f>
+        <f>VF($D$18; B37*12; -$D$17)</f>
         <v/>
       </c>
       <c r="E37" s="3">
@@ -840,7 +840,7 @@
         <v/>
       </c>
       <c r="D38" s="3">
-        <f>FV($D$18, B38*12, -$D$17)</f>
+        <f>VF($D$18; B38*12; -$D$17)</f>
         <v/>
       </c>
       <c r="E38" s="3">

</xml_diff>

<commit_message>
feat: implementa gráficos nativos no excel e gerador de pdf executivo para 3 perfis
</commit_message>
<xml_diff>
--- a/investment_simulator.xlsx
+++ b/investment_simulator.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,12 +50,6 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -72,8 +66,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="002B579A"/>
+        <bgColor rgb="002B579A"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +92,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,6 +170,281 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Distribuição da Carteira por Ativo</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'APP'!D23</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'APP'!$B$24:$B$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'APP'!$D$24:$D$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tipo de Investimento</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Aporte Alocado (R$)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Projeção de Patrimônio Acumulado (Longo Prazo)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'APP'!D33</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'APP'!$B$34:$B$38</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'APP'!$D$34:$D$38</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Anos</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Patrimônio (R$)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -467,17 +736,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="B2:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="69" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
-    <col width="69" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -485,12 +746,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -529,8 +784,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -568,12 +821,10 @@
         </is>
       </c>
       <c r="D18" s="7">
-        <f>SOMAPRODUTO(C24:C29; E24:E29) / 12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20"/>
+        <f>SOMARPRODUTO(C24:C29; E24:E29) / 12</f>
+        <v/>
+      </c>
+    </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -581,7 +832,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="B23" s="8" t="inlineStr">
         <is>
@@ -733,7 +983,6 @@
         <v/>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -855,6 +1104,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -866,14 +1116,6 @@
   </sheetPr>
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">

</xml_diff>